<commit_message>
Move visual to its own notebook
</commit_message>
<xml_diff>
--- a/interim/cluster_review.xlsx
+++ b/interim/cluster_review.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10510"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10517"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/ilya/chat-geospatial/interim/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C19A4771-FE97-8445-9B45-D5430365B466}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B49DE90-090F-7F4B-B76E-F76540D877A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="14060" yWindow="600" windowWidth="33480" windowHeight="26900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3869,7 +3869,7 @@
         <v>354</v>
       </c>
       <c r="G66" s="5" t="s">
-        <v>527</v>
+        <v>407</v>
       </c>
       <c r="H66" s="7" t="s">
         <v>355</v>

</xml_diff>